<commit_message>
fix: product_research finalize_node 重试逻辑修复（json_mode 缺 json 关键词导致 400）
</commit_message>
<xml_diff>
--- a/backend/generated_xlsx/Nike_20260710_预算流程回报分析.xlsx
+++ b/backend/generated_xlsx/Nike_20260710_预算流程回报分析.xlsx
@@ -286,7 +286,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>预算分配占比（50.0万）</a:t>
+              <a:t>预算分配占比（800.0万）</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -305,12 +305,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'预算总览'!$B$4:$B$8</f>
+              <f>'预算总览'!$B$4:$B$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'预算总览'!$C$4:$C$8</f>
+              <f>'预算总览'!$C$4:$C$9</f>
             </numRef>
           </val>
         </ser>
@@ -358,7 +358,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'预算明细'!B19</f>
+              <f>'预算明细'!B23</f>
             </strRef>
           </tx>
           <spPr>
@@ -371,12 +371,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'预算明细'!$A$20:$A$24</f>
+              <f>'预算明细'!$A$24:$A$29</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'预算明细'!$B$20:$B$24</f>
+              <f>'预算明细'!$B$24:$B$29</f>
             </numRef>
           </val>
         </ser>
@@ -675,7 +675,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'预期效果KPI'!B53</f>
+              <f>'预期效果KPI'!B52</f>
             </strRef>
           </tx>
           <spPr>
@@ -696,7 +696,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'预期效果KPI'!$B$54:$B$55</f>
+              <f>'预期效果KPI'!$B$53:$B$54</f>
             </numRef>
           </val>
         </ser>
@@ -777,7 +777,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'预期效果KPI'!B58</f>
+              <f>'预期效果KPI'!B57</f>
             </strRef>
           </tx>
           <spPr>
@@ -795,12 +795,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'预期效果KPI'!$A$59:$A$62</f>
+              <f>'预期效果KPI'!$A$58:$A$61</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'预期效果KPI'!$B$59:$B$62</f>
+              <f>'预期效果KPI'!$B$58:$B$61</f>
             </numRef>
           </val>
         </ser>
@@ -845,7 +845,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>12</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6480000" cy="5040000"/>
@@ -872,7 +872,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>22</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -926,7 +926,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="5040000"/>
@@ -948,7 +948,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6480000" cy="3600000"/>
@@ -970,7 +970,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>62</row>
+      <row>61</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="4320000"/>
@@ -1280,7 +1280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1299,7 +1299,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>上海营销方案XLSX数据</t>
+          <t>上海 单城市营销方案</t>
         </is>
       </c>
     </row>
@@ -1331,15 +1331,15 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>达人合作</t>
+          <t>盟域共建</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
@@ -1349,15 +1349,15 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>活动执行</t>
+          <t>赛事/活动</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>18</v>
+        <v>240</v>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>30.0%</t>
         </is>
       </c>
     </row>
@@ -1367,15 +1367,15 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>内容制作</t>
+          <t>达人合作</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>8</v>
+        <v>200</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>25.0%</t>
         </is>
       </c>
     </row>
@@ -1385,15 +1385,15 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>平台投放</t>
+          <t>内容运营</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>6</v>
+        <v>120</v>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
@@ -1403,46 +1403,64 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>运营资源</t>
+          <t>经营社联动</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>3</v>
+        <v>80</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="11" t="inlineStr">
+          <t>10.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>其他/预留</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>5.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="10" t="inlineStr"/>
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="C10" s="12" t="n">
+        <v>800</v>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>备注：总预算50万元，执行周期1个月，单城市上海，无版本对比。</t>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>备注：标准版预算总额 800 万元，所有金额单位：万元。单城市方案，无版本对比。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1455,7 +1473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1490,7 +1508,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>单版本(万元)</t>
+          <t>标准版(万元)</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -1502,349 +1520,503 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>达人合作</t>
+          <t>盟域共建</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>头部达人签约费</t>
+          <t>上海核心商圈快闪店</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>10位头部达人各1条品牌TVC拍摄+1场直播，签约费平均1.5万/条</t>
+          <t>在南京西路/淮海路等核心商圈搭建3个快闪体验空间，含搭建及运维</t>
         </is>
       </c>
       <c r="D3" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="E3" s="8" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>3个点位，每个约20万</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>达人合作</t>
+          <t>盟域共建</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>腰部达人佣金</t>
+          <t>联名主题门店改造</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>20位腰部达人视频佣金+GMV阶梯提成</t>
+          <t>与5家沪上潮店合作，进行Nike联名主题氛围改造与陈列更新</t>
         </is>
       </c>
       <c r="D4" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" s="8" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>5家门店，每家约8万</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>达人合作</t>
+          <t>盟域共建</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>尾部达人投放</t>
+          <t>城市运动地标打卡装置</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>50位尾部达人种草内容投放与激励</t>
+          <t>在外滩/徐汇滨江设置大型Nike运动地标装置，含审批与维护</t>
         </is>
       </c>
       <c r="D5" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" s="8" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>2个装置，含所有费用</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>活动执行</t>
+          <t>赛事/活动</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>主题训练营</t>
+          <t>『趁现在』城市接力跑（3场）</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>与10家健身工作室/瑜伽馆共建盟域，每月联合举办2场训练营</t>
+          <t>在上海世博园、世纪公园、东方体育中心举办3场主题跑步赛事</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" s="8" t="inlineStr"/>
+        <v>150</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>每场50万，含场地、物料、安保、奖金</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>活动执行</t>
+          <t>赛事/活动</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>城市定向赛</t>
+          <t>街头篮球挑战赛</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>每月1场定向赛，200人，赛事运营+路线设计+物资</t>
+          <t>在洛克公园等3处场地举办3v3篮球挑战赛，覆盖青少年及白领人群</t>
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="E7" s="8" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>3场，每场20万</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>活动执行</t>
+          <t>赛事/活动</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>夜跑派对</t>
+          <t>明星/意见领袖见面会</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>每月1场夜跑派对，500人，场地租赁+灯光音响+补给</t>
+          <t>邀请Nike签约运动员/教练举办2场粉丝见面会及训练营</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E8" s="8" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>2场，每场15万</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>活动执行</t>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>达人合作</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>限定徽章/抽奖</t>
+          <t>头部KOL深度共创（3-5位）</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>定制活动限定徽章、抽奖奖品及品牌周边</t>
+          <t>与上海本地运动/潮流类头部KOL合作，产出3条品牌视频及社交媒体活动</t>
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E9" s="8" t="inlineStr"/>
+        <v>120</v>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>含制作及投流</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>内容制作</t>
+          <t>达人合作</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>TVC/短视频拍摄</t>
+          <t>腰尾部达人铺量（20位）</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>城市街拍风格TVC（1条）+ 多场景短视频（5条）</t>
+          <t>招募20位上海本地运动/生活类腰尾部KOC进行产品测评及多平台种草</t>
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="8" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>每位平均3万</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>内容制作</t>
+          <t>达人合作</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>图文/拍照素材</t>
+          <t>直播合作（5场）</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>专业摄影师拍摄准点地标穿搭图、产品细节图</t>
+          <t>与5位健身/潮牌主播合作直播带货及品牌内容直播</t>
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" s="8" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>5场次，每场4万</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>内容制作</t>
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>内容运营</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>UGC话题运营</t>
+          <t>短视频拍摄制作（15条）</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>话题#上海每一步都算数 #跑出你的轨迹 等推广与互动奖励</t>
+          <t>拍摄15条Nike上海城市主题短视频，含脚本、拍摄、后期</t>
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="8" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>每条4万</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>平台投放</t>
+          <t>内容运营</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>小红书/抖音投流</t>
+          <t>图文内容制作（30篇）</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>精准投放上海18-35岁运动/时尚人群，持续4周</t>
+          <t>制作30篇小红书/微信图文种草内容，含设计及KOL合作嵌出</t>
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E13" s="8" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>每篇1万</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>运营资源</t>
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>内容运营</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>社群运营</t>
+          <t>官方账号运营与优化</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>跑者社群日常运营、打卡挑战、积分兑换</t>
+          <t>Nike上海本地官方双微一抖三个月内容规划、发布及互动维护</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" s="8" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>含人员及第三方工具</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>运营资源</t>
+          <t>经营社联动</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>数据监测/乐捐</t>
+          <t>门店引流活动（20场）</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>专属链接、折扣码追踪系统及数据分析工具</t>
+          <t>在20家Nike上海门店举办周末小型运动体验/产品沙龙，促进UGC</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="8" t="inlineStr"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
+        <v>40</v>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>每家门店2场次，每场1万</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
+          <t>经营社联动</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>会员专属社群运营</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>维护5个Nike上海会员社群，发布专属福利、活动及积分任务</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>3个月运营费</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>经营社联动</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>异业联动优惠券包</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>与10家上海本地餐饮/健身场馆合作，提供Nike顾客专属折扣券</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>含洽谈及系统对接</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>其他/预留</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>应急备用金</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>用于活动临时追加或者突发状况</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>其他/预留</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>数据监测与复盘</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>用于第三方数据监测、报告制作及复盘费用</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr"/>
-      <c r="C16" s="10" t="inlineStr"/>
-      <c r="D16" s="12" t="n">
-        <v>72</v>
-      </c>
-      <c r="E16" s="12" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr"/>
+      <c r="C20" s="10" t="inlineStr"/>
+      <c r="D20" s="12" t="n">
+        <v>800</v>
+      </c>
+      <c r="E20" s="12" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>费用大类</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>单版本(万)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>达人合作</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>活动执行</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>内容制作</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>平台投放</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="n">
-        <v>6</v>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>标准版(万)</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>运营资源</t>
+          <t>盟域共建</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>3</v>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>赛事/活动</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>达人合作</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>内容运营</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>经营社联动</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>其他/预留</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1877,7 +2049,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>活动流程 — 1个月执行时间线</t>
+          <t>活动流程 — 3个月执行时间线</t>
         </is>
       </c>
     </row>
@@ -1926,32 +2098,32 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>第1周</t>
+          <t>第1-2周</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>完成前期准备与资源整合</t>
+          <t>完成所有活动执行方案审批、场地预定与物料制作确认。</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>头部达人签约及TVC/短视频拍摄制作完成</t>
+          <t>完成快闪店、跑步赛、篮球赛等核心活动场地确认与合同签署</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>对接头部达人团队，确认创意脚本，进行TVC拍摄并完成后期剪辑</t>
+          <t>与南京西路、洛克公园等场地管理方对接，完成场地审批及安全备案</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>品牌部+媒介</t>
+          <t>盟域共建组</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>TVC成品1条+短视频5条</t>
+          <t>场地确认函、合同扫描件</t>
         </is>
       </c>
     </row>
@@ -1963,32 +2135,32 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>第1周</t>
+          <t>第1-2周</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>完成前期准备与资源整合</t>
+          <t>完成所有活动执行方案审批、场地预定与物料制作确认。</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>盟域场地确认与训练营排期制定</t>
+          <t>完成3位头部KOL及10位腰尾部达人合作意向确认及条款签订</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>与上海10家健身/瑜伽/篮球场馆签订合作协议，确定</t>
+          <t>通过MCN机构及直接邀约，发送Brief并确认合作人选及排期</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>市场活动部</t>
+          <t>达人合作组</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>场地合同+训练营排期表</t>
+          <t>合作备忘录、Brief</t>
         </is>
       </c>
     </row>
@@ -2000,32 +2172,32 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>第1周</t>
+          <t>第1-2周</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>完成前期准备与资源整合</t>
+          <t>完成所有活动执行方案审批、场地预定与物料制作确认。</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>启动城市跑者达人招募与社群搭建</t>
+          <t>完成15条短视频脚本定稿及拍摄前准备</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>发布上海本地跑者达人招募令，建立专属跑者微信群/企微社群</t>
+          <t>创意团队进行3轮脚本打磨，确定拍摄场地、艺人及服化道</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>社群运营部</t>
+          <t>内容运营组</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>招募信息+社群二维码</t>
+          <t>短视频脚本、拍摄日程表</t>
         </is>
       </c>
     </row>
@@ -2037,32 +2209,32 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>第1周</t>
+          <t>第1-2周</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>完成前期准备与资源整合</t>
+          <t>完成所有活动执行方案审批、场地预定与物料制作确认。</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>上线#上海每一步都算数 话题页</t>
+          <t>完成Nike官方上海双微一抖账号内容规划（前3周）</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>在小红书、抖音创建话题页面，设计话题规则与激励奖品</t>
+          <t>制定社媒日历，准备好种草图文和互动内容素材</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>内容运营</t>
+          <t>经营社联动组</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>话题页链接+活动规则文档</t>
+          <t>内容日历、素材库</t>
         </is>
       </c>
     </row>
@@ -2074,32 +2246,32 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>第2周</t>
+          <t>第3-4周</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>制造悬念与第一波传播</t>
+          <t>制造悬念与话题，吸引目标人群关注并有效沉淀。</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>腰部达人发布产品测评与穿搭视频</t>
+          <t>释放城市运动地标装置渲染图及快闪店效果图</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>20位腰部达人分别发布2条视频（测评与穿搭），附专属折扣码</t>
+          <t>在社交平台分发悬念海报，联合KOL进行预告转发</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>媒介部+达人管理</t>
+          <t>盟域共建组</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>40条推广视频</t>
+          <t>悬念海报、KOL转发截图</t>
         </is>
       </c>
     </row>
@@ -2111,32 +2283,32 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>第2周</t>
+          <t>第3-4周</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>制造悬念与第一波传播</t>
+          <t>制造悬念与话题，吸引目标人群关注并有效沉淀。</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>举办第一场盟域主题训练营</t>
+          <t>启动首轮腰部KOC铺量，产出20篇图文种草</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>在上海中心区域（如静安寺附近）健身工作室举办Nike Move晨跑+HIIT训练营</t>
+          <t>向20位KOC寄送产品，跟踪内容生产进度并审核</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>市场活动部</t>
+          <t>达人合作组</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>参与人数60人+活动图文</t>
+          <t>20篇小红书/微信推文</t>
         </is>
       </c>
     </row>
@@ -2148,32 +2320,32 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>第2周</t>
+          <t>第3-4周</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>制造悬念与第一波传播</t>
+          <t>制造悬念与话题，吸引目标人群关注并有效沉淀。</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>城市定向赛报名注册开启</t>
+          <t>发布第一条头部KOL共创品牌短视频</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>通过小程序/APP发布定向赛报名链接，限量200人</t>
+          <t>协调KOL拍摄剪辑，在抖音/B站首发，并匹配dou+推流</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>赛事运营</t>
+          <t>内容运营组</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>报名页面+报名数据</t>
+          <t>上线1条优质视频</t>
         </is>
       </c>
     </row>
@@ -2185,32 +2357,32 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>第2周</t>
+          <t>第3-4周</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>制造悬念与第一波传播</t>
+          <t>制造悬念与话题，吸引目标人群关注并有效沉淀。</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>平台投流第一期启动</t>
+          <t>上线报名H5页面，开启城市接力跑与街头篮球赛报名</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>针对上海地区18-35岁运动兴趣人群，定向投放TVC预告片与达人视频</t>
+          <t>通过Nike官方小程序及合作KOL二维码渠道开放名额</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>效果投放</t>
+          <t>赛事/活动组</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>曝光100万+互动5万+</t>
+          <t>报名页面、报名用户数据</t>
         </is>
       </c>
     </row>
@@ -2222,32 +2394,32 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>第3周</t>
+          <t>第5-9周</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>集中引爆线下活动与线上互动</t>
+          <t>通过高频、高互动活动引爆声量与销量。</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>举办城市定向赛（200人）</t>
+          <t>连续举办3场城市接力跑 + 3场街头篮球挑战赛</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>在外滩-徐汇滨江路线完成定向赛，打卡点设置装备体验与抽奖</t>
+          <t>按照筹备计划执行6场活动，确保物料、安保、媒体拍摄到位</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>赛事运营+品牌部</t>
+          <t>赛事/活动组</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>200人完赛+活动视频/图片</t>
+          <t>6场活动照片/视频、参与人次</t>
         </is>
       </c>
     </row>
@@ -2259,32 +2431,32 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>第3周</t>
+          <t>第5-9周</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>集中引爆线下活动与线上互动</t>
+          <t>通过高频、高互动活动引爆声量与销量。</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>举办夜跑派对（500人）</t>
+          <t>核心商圈快闪店及联名主题门店正式营业</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>在世纪公园/徐汇滨江举办夜跑派对，设置DJ、补给站、限定徽章</t>
+          <t>配合活动制造线下人流，在快闪店举办小型签售/教练指导</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>市场活动部</t>
+          <t>盟域共建组</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>500人参与+直播曝光</t>
+          <t>快闪店照片、门店销售额</t>
         </is>
       </c>
     </row>
@@ -2296,32 +2468,32 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>第3周</t>
+          <t>第5-9周</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>集中引爆线下活动与线上互动</t>
+          <t>通过高频、高互动活动引爆声量与销量。</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>尾部达人集中发布种草内容</t>
+          <t>头部KOL第二轮+ 5场直播带货密集上线</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>50位尾部达人同步发布图文/短视频种草，引导社群打卡</t>
+          <t>KOL直播+达人合作内容，重点推广当季Nike跑鞋及篮球鞋</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>媒介部</t>
+          <t>达人合作组</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>50条种草内容</t>
+          <t>直播片段、销售数据</t>
         </is>
       </c>
     </row>
@@ -2333,32 +2505,32 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>第3周</t>
+          <t>第5-9周</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>集中引爆线下活动与线上互动</t>
+          <t>通过高频、高互动活动引爆声量与销量。</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>社群打卡挑战启动</t>
+          <t>每周发布2-3条城市主题短视频，保持线上热度</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>跑者社群发起每日跑步打卡，连续7天得限定奖牌</t>
+          <t>内容团队按计划产出以活动为素材的短视频，配合官方账号发布</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>社群运营</t>
+          <t>内容运营组</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>社群活跃度提升30%</t>
+          <t>15条短视频上线</t>
         </is>
       </c>
     </row>
@@ -2370,32 +2542,32 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>第4周</t>
+          <t>第10-12周</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>促进销售转化与活动收官</t>
+          <t>持续收割流量，推动销售转化并沉淀品牌资产。</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>上线限时折扣与拼团活动</t>
+          <t>优惠券组合及异业联动合作上线，引导到店消费</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>推出新款跑鞋限时8折、3人成团7.5折，专属折扣码有效</t>
+          <t>与餐饮/健身店合作发放Nike专属券，引导至门店核销</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>电商运营</t>
+          <t>经营社联动组</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>销售额达到80万</t>
+          <t>核销数据</t>
         </is>
       </c>
     </row>
@@ -2407,32 +2579,32 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>第4周</t>
+          <t>第10-12周</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>促进销售转化与活动收官</t>
+          <t>持续收割流量，推动销售转化并沉淀品牌资产。</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>收官活动：线上跑者大会</t>
+          <t>明星/意见领袖见面会举办，强化品牌专业度</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>邀请头部达人+优秀UGC用户直播分享跑步故事与装备体验</t>
+          <t>邀请签约运动员进行2场线下训练营及粉丝签名会</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>品牌部+媒介</t>
+          <t>赛事/活动组</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>直播观看50万+</t>
+          <t>线下活动参与人次</t>
         </is>
       </c>
     </row>
@@ -2444,32 +2616,32 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>第4周</t>
+          <t>第10-12周</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>促进销售转化与活动收官</t>
+          <t>持续收割流量，推动销售转化并沉淀品牌资产。</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>发奖与积分兑换</t>
+          <t>精选前几周优质UGC与PGC，进行二次传播</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>统计打卡挑战完成用户，发放限定奖牌与Nike会员积分</t>
+          <t>剪辑活动高光视频，主推用户测评内容及销量战报</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>社群运营</t>
+          <t>内容运营组</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>500枚奖牌寄出</t>
+          <t>总结视频、长图</t>
         </is>
       </c>
     </row>
@@ -2481,32 +2653,32 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>第4周</t>
+          <t>第10-12周</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>促进销售转化与活动收官</t>
+          <t>持续收割流量，推动销售转化并沉淀品牌资产。</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>数据复盘与报告</t>
+          <t>输出全案数据报告，复盘KPI达成情况</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>汇总曝光、互动、线索、转化、销售额数据，制作结案报告</t>
+          <t>汇总所有渠道数据，完成营销复盘报告并举办内部分享</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>数据分析+品牌部</t>
+          <t>项目负责人</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>结案PPT+Excel数据表</t>
+          <t>完整复盘报告PPT</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2735,7 @@
         <v>5</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -2573,10 +2745,10 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2594,7 +2766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2631,7 +2803,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>单版本目标值</t>
+          <t>标准版目标值</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -2641,7 +2813,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>单版本数值</t>
+          <t>标准版数值</t>
         </is>
       </c>
     </row>
@@ -2653,26 +2825,26 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>总曝光量</t>
+          <t>整体曝光量（人次）</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>全渠道曝光量（含流量、自有渠道、达人内容自然曝光）</t>
+          <t>线上线下总曝光人次</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>500万次</t>
+          <t>1.5亿</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>曝光数据</t>
+          <t>程序化采买+自然曝光</t>
         </is>
       </c>
       <c r="G3" s="9" t="n">
-        <v>500</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -2683,26 +2855,26 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>UGC话题量</t>
+          <t>社交声量（互动量）</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>#上海每一步都算数 话题下新增UGC内容数</t>
+          <t>微博/抖音/小红书总互动事件数（转评赞）</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1万条</t>
+          <t>500万</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>话题页数据</t>
+          <t>KOL+UGC</t>
         </is>
       </c>
       <c r="G4" s="9" t="n">
-        <v>10000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
@@ -2713,26 +2885,26 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>达人内容互动量</t>
+          <t>品牌搜索指数提升率</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>达人视频/图文的总点赞+评论+分享</t>
+          <t>百度/微信指数较活动前增长率</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>20万次</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>互动数据</t>
+          <t>内容优化+SEO</t>
         </is>
       </c>
       <c r="G5" s="9" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -2743,26 +2915,26 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>品牌搜索指数提升</t>
+          <t>PR媒体报道数量</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>上海地区Nike关键词搜索量环比增幅</t>
+          <t>获得主流媒体/垂媒报道篇数</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>50篇</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>搜索指数</t>
+          <t>媒体合作</t>
         </is>
       </c>
       <c r="G6" s="9" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -2773,26 +2945,26 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>新用户登录/注册</t>
+          <t>官方私域新增粉丝（全渠道）</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>通过专属链接注册成为Nike会员的新用户数</t>
+          <t>Nike上海区域公众号/小程序/微信社群新增粉丝数</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1.5万</t>
+          <t>20万</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>CRM数据</t>
+          <t>小程序引流+活动关注</t>
         </is>
       </c>
       <c r="G7" s="9" t="n">
-        <v>15000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
@@ -2803,26 +2975,26 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>跑者社群成员数</t>
+          <t>活动参与人次</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>活动期间新增社群成员</t>
+          <t>线下活动（快闪、比赛、见面会）总参与人次</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>800人</t>
+          <t>8万</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>社群数据</t>
+          <t>活动互动</t>
         </is>
       </c>
       <c r="G8" s="9" t="n">
-        <v>800</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -2833,26 +3005,26 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>训练营/赛事参与人数</t>
+          <t>UGC内容产出量</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>活动期间所有线下活动总参与人次</t>
+          <t>用户自发产出的图文/短视频内容量</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>2000人次</t>
+          <t>3000条</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>活动数据</t>
+          <t>激励任务</t>
         </is>
       </c>
       <c r="G9" s="9" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
@@ -2863,26 +3035,26 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>小红书/抖音粉丝增长</t>
+          <t>报名H5页面留资量</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>品牌官方账号在上海地区新增粉丝数</t>
+          <t>填写报名信息的有效用户数</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>1.5万</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>平台数据</t>
+          <t>赛事报名</t>
         </is>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
@@ -2893,26 +3065,26 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>专属链接/折扣码销售额</t>
+          <t>线上GMV（万元）</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>通过专属链接或折扣码产生的订单总额</t>
+          <t>Nike天猫/京东旗舰店上海区域销售额</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>80万元</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>电商后台数据</t>
+          <t>直播+DTC</t>
         </is>
       </c>
       <c r="G11" s="9" t="n">
-        <v>80</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -2923,26 +3095,26 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>转化率</t>
+          <t>线下门店销售额（万元）</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>点击专属链接到达商品页的访客中完成购买的比例</t>
+          <t>上海区域20家核心门店活动期间总销售额</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>转化漏斗数据</t>
+          <t>门店引流</t>
         </is>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
@@ -2953,26 +3125,26 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>线索数</t>
+          <t>新客转化率</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>通过活动表单/小程序提交的用户信息（如试穿预约、咨询）</t>
+          <t>新增粉丝中转化为购买用户的比例</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>1.5万条</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>线索管理系统</t>
+          <t>优惠券</t>
         </is>
       </c>
       <c r="G13" s="9" t="n">
-        <v>15000</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
@@ -2983,26 +3155,26 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>复购意向率</t>
+          <t>领券核销率</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>活动后7天内社群内表达复购意愿的用户占比</t>
+          <t>发放异业联名优惠券的核销比例</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>社群调查</t>
+          <t>到店核销</t>
         </is>
       </c>
       <c r="G14" s="9" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
@@ -3013,26 +3185,26 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>线下盟域合作场馆数</t>
+          <t>快闪店/主题店数量</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>达成长期合作的健身/瑜伽/篮球场馆数量</t>
+          <t>合作搭建的快闪与主题门店数量</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>10家</t>
+          <t>8家</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>合作合同</t>
+          <t>盟域共建</t>
         </is>
       </c>
       <c r="G15" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
@@ -3043,26 +3215,26 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>线上达人合作人数</t>
+          <t>异业合作门店数量</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>活动期间签约并完成内容的达人总数</t>
+          <t>达成合作的异业门店数（餐饮/健身）</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>80人</t>
+          <t>10家</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>达人管理平台</t>
+          <t>经营社联动</t>
         </is>
       </c>
       <c r="G16" s="9" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
@@ -3073,209 +3245,197 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>经营社体验区覆盖</t>
+          <t>社交平台店铺矩阵建设</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>在上海线下门店/体验区设置的互动展陈覆盖数</t>
+          <t>在抖音/小红书/微信小程序完成店铺开设或优化</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>5个</t>
+          <t>3个平台</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>门店数据</t>
+          <t>内容运营</t>
         </is>
       </c>
       <c r="G17" s="9" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>渠道建设</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>自有渠道引流</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>从活动页/社群引导至官方APP/小程序的用户数</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>2万人</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>自有渠道数据</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="n">
-        <v>20000</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>ROI 投入产出分析</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>ROI 投入产出分析</t>
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>总投入</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>万元</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>活动总预算</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>800.0</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>标准版</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>总投入（万元）</t>
+          <t>预估总产出</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>项目总预算</t>
+          <t>万元</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>所有费用类别之和</t>
+          <t>线上+线下GMV总和</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr"/>
+          <t>3200.0</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>线上2000+线下1200</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>预估营收（万元）</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>来自专属链接的销售额</t>
-        </is>
-      </c>
+          <t>预估ROI</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr"/>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>直接归因成交额</t>
+          <t>产出/投入</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr"/>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>ROI</t>
+          <t>效率</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>投入产出比</t>
+          <t>元/曝光</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>营收/投入</t>
+          <t>总预算/总曝光人次（万）</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>1.6</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr"/>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>单用户获取成本（元）</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>CPA</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>总预算/新用户数</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>33.3</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>50万/1.5万</t>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>换算后</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>标准版</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>项目</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>单版本</t>
-        </is>
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>总预算（万元）</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="n">
+        <v>800</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>总投入</t>
+          <t>预估营收（万元）</t>
         </is>
       </c>
       <c r="B54" s="19" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>预估营收</t>
-        </is>
-      </c>
-      <c r="B55" s="19" t="n">
-        <v>80</v>
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>维度</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>标准版得分</t>
+        </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>维度</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>单版本得分</t>
-        </is>
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>品牌传播</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>品牌传播</t>
+          <t>用户增长</t>
         </is>
       </c>
       <c r="B59" s="7" t="n">
@@ -3285,37 +3445,27 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>用户增长</t>
+          <t>销售转化</t>
         </is>
       </c>
       <c r="B60" s="7" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>销售转化</t>
+          <t>渠道建设</t>
         </is>
       </c>
       <c r="B61" s="7" t="n">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
-        <is>
-          <t>渠道建设</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A19:E19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>